<commit_message>
feat: template abastecimentos — adiciona colunas Hodometro e Horimetro
</commit_message>
<xml_diff>
--- a/estudo-de-rede/template_abastecimentos_fni.xlsx
+++ b/estudo-de-rede/template_abastecimentos_fni.xlsx
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P105"/>
+  <dimension ref="A1:R105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -545,11 +545,31 @@
           <t>FNI Gestão de Frotas — Template de Abastecimentos</t>
         </is>
       </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Hodometro</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Horimetro</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>⚠️ Campos obrigatórios estão marcados com *. Não altere os nomes das colunas. Salve como .xlsx antes de fazer o upload.</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Leitura do hodômetro (km) no momento do abastecimento. Ex: 125000</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Leitura do horímetro (horas) para veículos como tratores. Ex: 4500.5</t>
         </is>
       </c>
     </row>

</xml_diff>